<commit_message>
#4 Design In Progress
</commit_message>
<xml_diff>
--- a/(Updated) BOM_CB_BIU_S2v2.0_Changes.xlsx
+++ b/(Updated) BOM_CB_BIU_S2v2.0_Changes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eSpark-Consultants\robertMeares-VCU-BCU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96856975-7215-4A9F-BD7C-AFAC2A64436F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13990789-0E4C-4A63-BC98-C01D96B4FB5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="979" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="542">
   <si>
     <t>C1,C142</t>
   </si>
@@ -1659,6 +1659,12 @@
   </si>
   <si>
     <t>91302-32-067R2B (M2 Connector)</t>
+  </si>
+  <si>
+    <t>DT1240-04LP-7</t>
+  </si>
+  <si>
+    <t>Reference schematic used</t>
   </si>
 </sst>
 </file>
@@ -4389,14 +4395,14 @@
         <v>0.15</v>
       </c>
       <c r="P33" s="11">
-        <f t="shared" ref="P33:P64" si="4">O33*B33</f>
+        <f t="shared" ref="P33:P53" si="4">O33*B33</f>
         <v>1.05</v>
       </c>
       <c r="Q33" s="11">
         <v>2.8000000000000001E-2</v>
       </c>
       <c r="R33" s="11">
-        <f t="shared" ref="R33:R64" si="5">Q33*B33</f>
+        <f t="shared" ref="R33:R53" si="5">Q33*B33</f>
         <v>0.19600000000000001</v>
       </c>
       <c r="S33" s="11">
@@ -4404,7 +4410,7 @@
         <v>1.1200000000000002E-2</v>
       </c>
       <c r="T33" s="11">
-        <f t="shared" ref="T33:T64" si="7">S33*B33</f>
+        <f t="shared" ref="T33:T53" si="7">S33*B33</f>
         <v>7.8400000000000011E-2</v>
       </c>
     </row>
@@ -7664,7 +7670,7 @@
         <v>2.0000000000000004E-2</v>
       </c>
       <c r="T87" s="11">
-        <f t="shared" ref="T87:T118" si="12">S87*B87</f>
+        <f t="shared" ref="T87:T117" si="12">S87*B87</f>
         <v>4.0000000000000008E-2</v>
       </c>
     </row>
@@ -8413,8 +8419,12 @@
       <c r="G100" s="5" t="s">
         <v>417</v>
       </c>
-      <c r="H100" s="42"/>
-      <c r="I100" s="42"/>
+      <c r="H100" s="42" t="s">
+        <v>540</v>
+      </c>
+      <c r="I100" s="42" t="s">
+        <v>541</v>
+      </c>
       <c r="J100" s="5" t="s">
         <v>419</v>
       </c>

</xml_diff>

<commit_message>
#4 16 of 19 Done
</commit_message>
<xml_diff>
--- a/(Updated) BOM_CB_BIU_S2v2.0_Changes.xlsx
+++ b/(Updated) BOM_CB_BIU_S2v2.0_Changes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eSpark-Consultants\robertMeares-VCU-BCU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13990789-0E4C-4A63-BC98-C01D96B4FB5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66CC8782-0140-45AE-A777-E13A360CD870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CARRIER_BOARD_S2_V2.0" sheetId="1" r:id="rId1"/>
@@ -1628,9 +1628,6 @@
     <t>CBR04C229B5GACAUTO</t>
   </si>
   <si>
-    <t>PESD2CANFD27LT-QR</t>
-  </si>
-  <si>
     <t>lxora default assembly part</t>
   </si>
   <si>
@@ -1665,6 +1662,9 @@
   </si>
   <si>
     <t>Reference schematic used</t>
+  </si>
+  <si>
+    <t>DESD2CAN2SOQ-7</t>
   </si>
 </sst>
 </file>
@@ -4437,7 +4437,7 @@
         <v>131</v>
       </c>
       <c r="H34" s="42" t="s">
-        <v>529</v>
+        <v>541</v>
       </c>
       <c r="I34" s="42" t="s">
         <v>513</v>
@@ -5228,7 +5228,7 @@
         <v>69307101081</v>
       </c>
       <c r="I47" s="42" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="J47" s="5" t="s">
         <v>86</v>
@@ -5933,10 +5933,10 @@
         <v>243</v>
       </c>
       <c r="H59" s="42" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I59" s="42" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="J59" s="5" t="s">
         <v>245</v>
@@ -6057,10 +6057,10 @@
         <v>252</v>
       </c>
       <c r="H61" s="42" t="s">
+        <v>534</v>
+      </c>
+      <c r="I61" s="42" t="s">
         <v>535</v>
-      </c>
-      <c r="I61" s="42" t="s">
-        <v>536</v>
       </c>
       <c r="J61" s="5" t="s">
         <v>86</v>
@@ -7939,10 +7939,10 @@
         <v>383</v>
       </c>
       <c r="H92" s="42" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="I92" s="42" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="J92" s="5" t="s">
         <v>384</v>
@@ -8070,7 +8070,7 @@
         <v>508</v>
       </c>
       <c r="I94" s="42" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="J94" s="5" t="s">
         <v>395</v>
@@ -8134,7 +8134,7 @@
         <v>511</v>
       </c>
       <c r="I95" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="J95" s="5" t="s">
         <v>401</v>
@@ -8420,10 +8420,10 @@
         <v>417</v>
       </c>
       <c r="H100" s="42" t="s">
+        <v>539</v>
+      </c>
+      <c r="I100" s="42" t="s">
         <v>540</v>
-      </c>
-      <c r="I100" s="42" t="s">
-        <v>541</v>
       </c>
       <c r="J100" s="5" t="s">
         <v>419</v>
@@ -8544,10 +8544,10 @@
         <v>429</v>
       </c>
       <c r="H102" s="42" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="I102" s="42" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="J102" s="5" t="s">
         <v>86</v>

</xml_diff>

<commit_message>
#4 Complete - Without Top Sheet, LTE M2 module, Audio Circuit
</commit_message>
<xml_diff>
--- a/(Updated) BOM_CB_BIU_S2v2.0_Changes.xlsx
+++ b/(Updated) BOM_CB_BIU_S2v2.0_Changes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eSpark-Consultants\robertMeares-VCU-BCU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66CC8782-0140-45AE-A777-E13A360CD870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0142A9E-85DB-413B-AB2E-DBF6B6D24361}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1574,9 +1574,6 @@
     <t>Crystal</t>
   </si>
   <si>
-    <t>ISO1042QDWRQ1</t>
-  </si>
-  <si>
     <t>GRT188R61C106KE13D</t>
   </si>
   <si>
@@ -1665,6 +1662,9 @@
   </si>
   <si>
     <t>DESD2CAN2SOQ-7</t>
+  </si>
+  <si>
+    <t>ADM3057EBRWZ</t>
   </si>
 </sst>
 </file>
@@ -2689,10 +2689,10 @@
         <v>31</v>
       </c>
       <c r="H6" s="42" t="s">
+        <v>511</v>
+      </c>
+      <c r="I6" s="42" t="s">
         <v>512</v>
-      </c>
-      <c r="I6" s="42" t="s">
-        <v>513</v>
       </c>
       <c r="J6" s="5">
         <v>603</v>
@@ -2813,10 +2813,10 @@
         <v>37</v>
       </c>
       <c r="H8" s="42" t="s">
+        <v>513</v>
+      </c>
+      <c r="I8" s="42" t="s">
         <v>514</v>
-      </c>
-      <c r="I8" s="42" t="s">
-        <v>515</v>
       </c>
       <c r="J8" s="5">
         <v>805</v>
@@ -2877,10 +2877,10 @@
         <v>41</v>
       </c>
       <c r="H9" s="42" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="I9" s="42" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="J9" s="5">
         <v>1206</v>
@@ -2941,10 +2941,10 @@
         <v>45</v>
       </c>
       <c r="H10" s="42" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="I10" s="42" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J10" s="5">
         <v>1210</v>
@@ -3007,10 +3007,10 @@
         <v>50</v>
       </c>
       <c r="H11" s="42" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="I11" s="42" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J11" s="5">
         <v>1210</v>
@@ -3191,10 +3191,10 @@
         <v>60</v>
       </c>
       <c r="H14" s="42" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="I14" s="42" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="J14" s="5">
         <v>603</v>
@@ -3255,10 +3255,10 @@
         <v>64</v>
       </c>
       <c r="H15" s="42" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="I15" s="42" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J15" s="5">
         <v>603</v>
@@ -3319,10 +3319,10 @@
         <v>67</v>
       </c>
       <c r="H16" s="42" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="I16" s="42" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="J16" s="5">
         <v>1206</v>
@@ -3445,10 +3445,10 @@
         <v>74</v>
       </c>
       <c r="H18" s="42" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="I18" s="42" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J18" s="5">
         <v>1210</v>
@@ -3509,10 +3509,10 @@
         <v>77</v>
       </c>
       <c r="H19" s="42" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="I19" s="42" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J19" s="5">
         <v>603</v>
@@ -3573,10 +3573,10 @@
         <v>81</v>
       </c>
       <c r="H20" s="42" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="I20" s="42" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J20" s="5">
         <v>1206</v>
@@ -3637,10 +3637,10 @@
         <v>85</v>
       </c>
       <c r="H21" s="42" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="I21" s="42" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>86</v>
@@ -3885,10 +3885,10 @@
         <v>98</v>
       </c>
       <c r="H25" s="42" t="s">
+        <v>525</v>
+      </c>
+      <c r="I25" s="42" t="s">
         <v>526</v>
-      </c>
-      <c r="I25" s="42" t="s">
-        <v>527</v>
       </c>
       <c r="J25" s="5">
         <v>603</v>
@@ -4251,10 +4251,10 @@
         <v>118</v>
       </c>
       <c r="H31" s="42" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="I31" s="42" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="J31" s="5">
         <v>402</v>
@@ -4437,10 +4437,10 @@
         <v>131</v>
       </c>
       <c r="H34" s="42" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="I34" s="42" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J34" s="5" t="s">
         <v>132</v>
@@ -5228,7 +5228,7 @@
         <v>69307101081</v>
       </c>
       <c r="I47" s="42" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="J47" s="5" t="s">
         <v>86</v>
@@ -5933,10 +5933,10 @@
         <v>243</v>
       </c>
       <c r="H59" s="42" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="I59" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="J59" s="5" t="s">
         <v>245</v>
@@ -6057,10 +6057,10 @@
         <v>252</v>
       </c>
       <c r="H61" s="42" t="s">
+        <v>533</v>
+      </c>
+      <c r="I61" s="42" t="s">
         <v>534</v>
-      </c>
-      <c r="I61" s="42" t="s">
-        <v>535</v>
       </c>
       <c r="J61" s="5" t="s">
         <v>86</v>
@@ -7939,10 +7939,10 @@
         <v>383</v>
       </c>
       <c r="H92" s="42" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="I92" s="42" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="J92" s="5" t="s">
         <v>384</v>
@@ -8006,7 +8006,7 @@
         <v>506</v>
       </c>
       <c r="I93" s="42" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J93" s="5" t="s">
         <v>389</v>
@@ -8070,7 +8070,7 @@
         <v>508</v>
       </c>
       <c r="I94" s="42" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="J94" s="5" t="s">
         <v>395</v>
@@ -8131,10 +8131,10 @@
         <v>400</v>
       </c>
       <c r="H95" s="42" t="s">
-        <v>511</v>
+        <v>541</v>
       </c>
       <c r="I95" s="42" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="J95" s="5" t="s">
         <v>401</v>
@@ -8420,10 +8420,10 @@
         <v>417</v>
       </c>
       <c r="H100" s="42" t="s">
+        <v>538</v>
+      </c>
+      <c r="I100" s="42" t="s">
         <v>539</v>
-      </c>
-      <c r="I100" s="42" t="s">
-        <v>540</v>
       </c>
       <c r="J100" s="5" t="s">
         <v>419</v>
@@ -8544,10 +8544,10 @@
         <v>429</v>
       </c>
       <c r="H102" s="42" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="I102" s="42" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="J102" s="5" t="s">
         <v>86</v>
@@ -9704,7 +9704,7 @@
         <v>400</v>
       </c>
       <c r="G6" s="41" t="s">
-        <v>511</v>
+        <v>541</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>401</v>

</xml_diff>